<commit_message>
Replace real names/info with fake sample data across app, examples, tests, and docs
Co-authored-by: Copilot App <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/create-call-sheet/examples/sample_output.xlsx
+++ b/create-call-sheet/examples/sample_output.xlsx
@@ -68,13 +68,13 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00111111"/>
+      <color rgb="002563EB"/>
       <sz val="12"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00111111"/>
+      <color rgb="002563EB"/>
       <sz val="11"/>
     </font>
     <font>
@@ -682,7 +682,7 @@
     <row r="4" ht="26" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>GitHub × ASOS</t>
+          <t>Acme Widgets × Northwind</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
@@ -721,18 +721,18 @@
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>GitHub</t>
+          <t>Acme Widgets</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>MAJORITY</t>
+          <t>SAMPLE STUDIOS</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr"/>
       <c r="L6" s="5" t="inlineStr">
         <is>
-          <t>GH-2026-014</t>
+          <t>SAMPLE-2026-001</t>
         </is>
       </c>
     </row>
@@ -754,17 +754,17 @@
       <c r="E9" s="8" t="inlineStr">
         <is>
           <t>LOCATION
-Greater London House
-Hampstead Rd
-London NW1 7FB, United Kingdom</t>
+Sample House
+123 Example Rd
+London NW1 0AA, United Kingdom</t>
         </is>
       </c>
       <c r="J9" s="9" t="inlineStr">
         <is>
           <t>NEAREST HOSPITAL
-University College Hospital
-235 Euston Rd, London NW1 2BU
-020 3456 7890
+General Hospital
+1 Example Rd, London NW1 0BB
+020 0000 0000
 DIAL 911 IN EMERGENCY</t>
         </is>
       </c>
@@ -866,12 +866,12 @@
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>Limited street parking around Hampstead Rd. Loading at front, then park in NCP Euston Garage (5 min walk). Pay for the day.</t>
+          <t>Limited street parking nearby. Loading at front, then park in Example Garage (5 min walk). Pay for the day.</t>
         </is>
       </c>
       <c r="H19" s="14" t="inlineStr">
         <is>
-          <t>Reception is on Ground Floor. Sign in for Grace Beatty, badge to Floor 4. Loading dock around back via service road.</t>
+          <t>Reception is on Ground Floor. Sign in for Riley Stone, badge to Floor 4. Loading dock around back via service road.</t>
         </is>
       </c>
     </row>
@@ -919,7 +919,7 @@
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Alex Perrault</t>
+          <t>Jordan Rivers</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>+1 206-919-0160</t>
+          <t>+1 555-010-0100</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr"/>
@@ -939,7 +939,7 @@
     <row r="25" ht="22" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Cathleen Alexander</t>
+          <t>Morgan Blake</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
@@ -949,7 +949,7 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>+1 213-864-8680</t>
+          <t>+1 555-010-0101</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr"/>
@@ -1032,7 +1032,7 @@
       </c>
       <c r="K30" s="18" t="inlineStr">
         <is>
-          <t>Dylan Morley</t>
+          <t>Jamie Fox</t>
         </is>
       </c>
       <c r="M30" s="18" t="inlineStr"/>
@@ -1045,7 +1045,7 @@
       </c>
       <c r="C31" s="17" t="inlineStr">
         <is>
-          <t>INTERVIEW 1: Dylan Morley</t>
+          <t>INTERVIEW 1: Jamie Fox</t>
         </is>
       </c>
       <c r="H31" s="17" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="K31" s="17" t="inlineStr">
         <is>
-          <t>Dylan Morley</t>
+          <t>Jamie Fox</t>
         </is>
       </c>
       <c r="M31" s="17" t="inlineStr">
@@ -1082,7 +1082,7 @@
       </c>
       <c r="K32" s="18" t="inlineStr">
         <is>
-          <t>Lewis Holmes</t>
+          <t>Devon Cole</t>
         </is>
       </c>
       <c r="M32" s="18" t="inlineStr"/>
@@ -1095,7 +1095,7 @@
       </c>
       <c r="C33" s="17" t="inlineStr">
         <is>
-          <t>INTERVIEW 2: Lewis Holmes</t>
+          <t>INTERVIEW 2: Devon Cole</t>
         </is>
       </c>
       <c r="H33" s="17" t="inlineStr">
@@ -1105,7 +1105,7 @@
       </c>
       <c r="K33" s="17" t="inlineStr">
         <is>
-          <t>Lewis Holmes</t>
+          <t>Devon Cole</t>
         </is>
       </c>
       <c r="M33" s="17" t="inlineStr">
@@ -1145,7 +1145,7 @@
       </c>
       <c r="C35" s="17" t="inlineStr">
         <is>
-          <t>INTERVIEW 3: Przemek Czarnecki</t>
+          <t>INTERVIEW 3: Alex Kim</t>
         </is>
       </c>
       <c r="H35" s="17" t="inlineStr">
@@ -1155,7 +1155,7 @@
       </c>
       <c r="K35" s="17" t="inlineStr">
         <is>
-          <t>Przemek</t>
+          <t>Alex Kim</t>
         </is>
       </c>
       <c r="M35" s="17" t="inlineStr">
@@ -1182,7 +1182,7 @@
       </c>
       <c r="K36" s="18" t="inlineStr">
         <is>
-          <t>Chris Newark</t>
+          <t>Avery Reed</t>
         </is>
       </c>
       <c r="M36" s="18" t="inlineStr"/>
@@ -1195,7 +1195,7 @@
       </c>
       <c r="C37" s="17" t="inlineStr">
         <is>
-          <t>INTERVIEW 4: Chris Newark</t>
+          <t>INTERVIEW 4: Avery Reed</t>
         </is>
       </c>
       <c r="H37" s="17" t="inlineStr">
@@ -1205,7 +1205,7 @@
       </c>
       <c r="K37" s="17" t="inlineStr">
         <is>
-          <t>Chris Newark</t>
+          <t>Avery Reed</t>
         </is>
       </c>
       <c r="M37" s="17" t="inlineStr">
@@ -1327,22 +1327,22 @@
       </c>
       <c r="D45" s="21" t="inlineStr">
         <is>
-          <t>Alex Perrault</t>
+          <t>Jordan Rivers</t>
         </is>
       </c>
       <c r="F45" s="22" t="inlineStr">
         <is>
-          <t>he/him</t>
+          <t>they/them</t>
         </is>
       </c>
       <c r="G45" s="21" t="inlineStr">
         <is>
-          <t>+1 206-919-0160</t>
+          <t>+1 555-010-0100</t>
         </is>
       </c>
       <c r="I45" s="21" t="inlineStr">
         <is>
-          <t>evillollive@github.com</t>
+          <t>jordan.rivers@example.com</t>
         </is>
       </c>
       <c r="M45" s="22" t="inlineStr">
@@ -1359,12 +1359,12 @@
     <row r="46" ht="19" customHeight="1">
       <c r="A46" s="20" t="inlineStr">
         <is>
-          <t>Producer (Majority)</t>
+          <t>Producer (Sample Studios)</t>
         </is>
       </c>
       <c r="D46" s="21" t="inlineStr">
         <is>
-          <t>Cathleen Alexander</t>
+          <t>Morgan Blake</t>
         </is>
       </c>
       <c r="F46" s="22" t="inlineStr">
@@ -1374,12 +1374,12 @@
       </c>
       <c r="G46" s="21" t="inlineStr">
         <is>
-          <t>+1 213-864-8680</t>
+          <t>+1 555-010-0101</t>
         </is>
       </c>
       <c r="I46" s="21" t="inlineStr">
         <is>
-          <t>ca@majorityfilm.com</t>
+          <t>morgan.blake@example.com</t>
         </is>
       </c>
       <c r="M46" s="22" t="inlineStr">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="D48" s="21" t="inlineStr">
         <is>
-          <t>Brett Bollier</t>
+          <t>Casey Lin</t>
         </is>
       </c>
       <c r="F48" s="22" t="inlineStr">
@@ -1418,12 +1418,12 @@
       </c>
       <c r="G48" s="21" t="inlineStr">
         <is>
-          <t>+1 503-866-5518</t>
+          <t>+1 555-010-0102</t>
         </is>
       </c>
       <c r="I48" s="21" t="inlineStr">
         <is>
-          <t>brett.bollier@gmail.com</t>
+          <t>casey.lin@example.com</t>
         </is>
       </c>
       <c r="M48" s="22" t="inlineStr">
@@ -1452,18 +1452,18 @@
       </c>
       <c r="D50" s="21" t="inlineStr">
         <is>
-          <t>Al Rice</t>
+          <t>Sam Doe</t>
         </is>
       </c>
       <c r="F50" s="22" t="inlineStr"/>
       <c r="G50" s="21" t="inlineStr">
         <is>
-          <t>+44 7917 606621</t>
+          <t>+1 555-010-0103</t>
         </is>
       </c>
       <c r="I50" s="21" t="inlineStr">
         <is>
-          <t>al@alricelights.com</t>
+          <t>sam.doe@example.com</t>
         </is>
       </c>
       <c r="M50" s="22" t="inlineStr">
@@ -1485,18 +1485,18 @@
       </c>
       <c r="D51" s="21" t="inlineStr">
         <is>
-          <t>Declan Duffy</t>
+          <t>Robin Park</t>
         </is>
       </c>
       <c r="F51" s="22" t="inlineStr"/>
       <c r="G51" s="21" t="inlineStr">
         <is>
-          <t>+44 7470 366961</t>
+          <t>+1 555-010-0106</t>
         </is>
       </c>
       <c r="I51" s="21" t="inlineStr">
         <is>
-          <t>derrick@declannotderrick.com</t>
+          <t>robin.park@example.com</t>
         </is>
       </c>
       <c r="M51" s="22" t="inlineStr">
@@ -1525,18 +1525,18 @@
       </c>
       <c r="D53" s="21" t="inlineStr">
         <is>
-          <t>Dominic Skinner</t>
+          <t>Taylor Quinn</t>
         </is>
       </c>
       <c r="F53" s="22" t="inlineStr"/>
       <c r="G53" s="21" t="inlineStr">
         <is>
-          <t>+44 7747 648953</t>
+          <t>+1 555-010-0104</t>
         </is>
       </c>
       <c r="I53" s="21" t="inlineStr">
         <is>
-          <t>dominiccskinner@gmail.com</t>
+          <t>taylor.quinn@example.com</t>
         </is>
       </c>
       <c r="M53" s="22" t="inlineStr">
@@ -1560,23 +1560,23 @@
     <row r="55" ht="19" customHeight="1">
       <c r="A55" s="20" t="inlineStr">
         <is>
-          <t>GitHub</t>
+          <t>Acme Widgets</t>
         </is>
       </c>
       <c r="D55" s="21" t="inlineStr">
         <is>
-          <t>Grace Beatty</t>
+          <t>Riley Stone</t>
         </is>
       </c>
       <c r="F55" s="22" t="inlineStr"/>
       <c r="G55" s="21" t="inlineStr">
         <is>
-          <t>+34 675 628 689</t>
+          <t>+1 555-010-0105</t>
         </is>
       </c>
       <c r="I55" s="21" t="inlineStr">
         <is>
-          <t>gracebeatty@github.com</t>
+          <t>riley.stone@example.com</t>
         </is>
       </c>
       <c r="M55" s="22" t="inlineStr">
@@ -1601,7 +1601,7 @@
       </c>
       <c r="D57" s="21" t="inlineStr">
         <is>
-          <t>Chris Newark</t>
+          <t>Avery Reed</t>
         </is>
       </c>
       <c r="F57" s="22" t="inlineStr"/>
@@ -1622,7 +1622,7 @@
       </c>
       <c r="D58" s="21" t="inlineStr">
         <is>
-          <t>Lew Holmes</t>
+          <t>Devon Cole</t>
         </is>
       </c>
       <c r="F58" s="22" t="inlineStr"/>
@@ -1650,18 +1650,18 @@
       </c>
       <c r="D60" s="21" t="inlineStr">
         <is>
-          <t>SL Vision LTD</t>
+          <t>Example Camera Rental</t>
         </is>
       </c>
       <c r="F60" s="22" t="inlineStr"/>
       <c r="G60" s="21" t="inlineStr">
         <is>
-          <t>+44 207 720 6464</t>
+          <t>+1 555-010-0107</t>
         </is>
       </c>
       <c r="I60" s="21" t="inlineStr">
         <is>
-          <t>hire@slvision.co.uk</t>
+          <t>hire@example.com</t>
         </is>
       </c>
       <c r="M60" s="22" t="inlineStr"/>
@@ -1675,18 +1675,18 @@
       </c>
       <c r="D61" s="21" t="inlineStr">
         <is>
-          <t>Al Rice Lights</t>
+          <t>Sample Lighting Co</t>
         </is>
       </c>
       <c r="F61" s="22" t="inlineStr"/>
       <c r="G61" s="21" t="inlineStr">
         <is>
-          <t>+44 7917 606621</t>
+          <t>+1 555-010-0103</t>
         </is>
       </c>
       <c r="I61" s="21" t="inlineStr">
         <is>
-          <t>al@alricelights.com</t>
+          <t>lighting@example.com</t>
         </is>
       </c>
       <c r="M61" s="22" t="inlineStr"/>
@@ -1700,18 +1700,18 @@
       </c>
       <c r="D62" s="21" t="inlineStr">
         <is>
-          <t>Inszone Insurance</t>
+          <t>Example Insurance Co</t>
         </is>
       </c>
       <c r="F62" s="22" t="inlineStr"/>
       <c r="G62" s="21" t="inlineStr">
         <is>
-          <t>+1 562-307-8417</t>
+          <t>+1 555-010-0108</t>
         </is>
       </c>
       <c r="I62" s="21" t="inlineStr">
         <is>
-          <t>tinsua@inszoneins.com</t>
+          <t>insurance@example.com</t>
         </is>
       </c>
       <c r="M62" s="22" t="inlineStr"/>
@@ -1868,7 +1868,7 @@
     <row r="77" ht="20" customHeight="1">
       <c r="A77" s="23" t="inlineStr">
         <is>
-          <t>Allergies / dietary restrictions: flag to Cathleen by EOD Thursday.</t>
+          <t>Allergies / dietary restrictions: flag to the Producer by EOD Thursday.</t>
         </is>
       </c>
     </row>
@@ -1938,7 +1938,7 @@
       </c>
       <c r="F88" s="21" t="inlineStr">
         <is>
-          <t>GH-2026-014</t>
+          <t>SAMPLE-2026-001</t>
         </is>
       </c>
     </row>
@@ -1950,7 +1950,7 @@
       </c>
       <c r="F89" s="21" t="inlineStr">
         <is>
-          <t>ca@majorityfilm.com</t>
+          <t>billing@example.com</t>
         </is>
       </c>
     </row>
@@ -1962,7 +1962,7 @@
       </c>
       <c r="F90" s="21" t="inlineStr">
         <is>
-          <t>Majority Film, 1234 Sunset Blvd, Los Angeles CA 90026</t>
+          <t>Sample Studios, 100 Example Ave, Anytown CA 90000</t>
         </is>
       </c>
     </row>
@@ -1982,7 +1982,7 @@
     <row r="93" ht="18" customHeight="1">
       <c r="A93" s="24" t="inlineStr">
         <is>
-          <t>PRODUCTION REPORT  (fill in during/after shoot — optional)</t>
+          <t>PRODUCTION REPORT  (fill in during/after filming, optional)</t>
         </is>
       </c>
     </row>
@@ -2296,7 +2296,9 @@
     <mergeCell ref="G72:H72"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J9" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId3"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.3" right="0.3" top="0.3" bottom="0.3" header="0.5" footer="0.5"/>
@@ -2358,7 +2360,7 @@
     <row r="8" ht="18" customHeight="1">
       <c r="B8" s="27" t="inlineStr">
         <is>
-          <t>Anything in [ brackets ] is a placeholder — replace with shoot info.</t>
+          <t>Anything in [ brackets ] is a placeholder; replace with shoot info.</t>
         </is>
       </c>
     </row>
@@ -2392,7 +2394,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="B14" s="27" t="inlineStr">
         <is>
-          <t>Sunrise and sunset are pre-filled where possible. Weather is left blank — click the 'Check weather' link in the quick-info ribbon to look it up.</t>
+          <t>Sunrise and sunset are pre-filled where possible. Weather is left blank. Click the 'Check weather' link in the quick-info ribbon to look it up.</t>
         </is>
       </c>
     </row>

</xml_diff>